<commit_message>
Update template.xlsx, add template_range.xlsx and package-lock.json.bak
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\socrasteeze\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\socrasteeze\Documents\GitHub\snuggpro-inspector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F8EB534-BB93-48A3-BAB9-130C02EFA381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C20BCC-C8EA-4D73-89A0-60DEAC2EC818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2748" yWindow="3348" windowWidth="34764" windowHeight="11460" activeTab="3" xr2:uid="{A99C927A-33D9-4317-A0E9-157DA9D92934}"/>
+    <workbookView xWindow="1920" yWindow="1908" windowWidth="32148" windowHeight="15372" xr2:uid="{A99C927A-33D9-4317-A0E9-157DA9D92934}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="5" r:id="rId1"/>
@@ -18,12 +18,25 @@
     <sheet name="ElectricUsageGrid" sheetId="2" r:id="rId3"/>
     <sheet name="GasUsageGrid" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="63">
   <si>
     <t>Fuel</t>
   </si>
@@ -194,6 +207,24 @@
   </si>
   <si>
     <t>MeasureCostOverride</t>
+  </si>
+  <si>
+    <t>Path</t>
+  </si>
+  <si>
+    <t>Combined Savings</t>
+  </si>
+  <si>
+    <t>Pilot Plus</t>
+  </si>
+  <si>
+    <t>kW</t>
+  </si>
+  <si>
+    <t>Home Type</t>
+  </si>
+  <si>
+    <t>HVAC Type</t>
   </si>
 </sst>
 </file>
@@ -689,13 +720,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -743,77 +773,16 @@
   </cellStyles>
   <dxfs count="25">
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
     </dxf>
     <dxf>
       <fill>
@@ -890,6 +859,65 @@
       </fill>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="none">
           <fgColor theme="0" tint="-0.14999847407452621"/>
@@ -913,16 +941,19 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -938,37 +969,42 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F6A17860-09D2-46D3-A243-4CF3C35A9E56}" name="Table4" displayName="Table4" ref="A1:A2" totalsRowShown="0">
-  <autoFilter ref="A1:A2" xr:uid="{F6A17860-09D2-46D3-A243-4CF3C35A9E56}"/>
-  <tableColumns count="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F6A17860-09D2-46D3-A243-4CF3C35A9E56}" name="Table4" displayName="Table4" ref="A1:E2" totalsRowShown="0">
+  <autoFilter ref="A1:E2" xr:uid="{F6A17860-09D2-46D3-A243-4CF3C35A9E56}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{2A2039BB-4A17-4CE0-8339-B20D0CBE5F97}" name="AuditId"/>
+    <tableColumn id="2" xr3:uid="{242991A7-2282-4AD7-A901-9B777F947707}" name="Path"/>
+    <tableColumn id="3" xr3:uid="{D845DCF8-EA7E-4850-9DC9-DB47A247BABC}" name="Combined Savings"/>
+    <tableColumn id="4" xr3:uid="{54CCFE7B-E886-404D-BBED-7067F7E7FBAF}" name="Home Type"/>
+    <tableColumn id="5" xr3:uid="{F0AAF654-7FF5-4931-88F0-B7D5211D4784}" name="HVAC Type"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DF844518-2BF6-446A-A312-CEB862DCE28B}" name="Table1" displayName="Table1" ref="A1:R11" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6" tableBorderDxfId="20">
-  <autoFilter ref="A1:R11" xr:uid="{DF844518-2BF6-446A-A312-CEB862DCE28B}"/>
-  <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{1C0006D7-B99F-4704-908A-2CA80F2C4948}" name="AuditId" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{CC9645AE-FB6D-4AEE-80F7-3A498704D7AE}" name="Measure" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{61A9A28F-0DC7-4361-B3A0-86A213988794}" name="Src" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{FE306C0E-B210-4780-8F5C-9021F0A2B9A0}" name="ReportingCode" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{8E31AB8D-C308-426E-B4B5-FEDE3ACE3234}" name="Code" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{E78062F7-BD26-4033-A7AE-088E604FD3BA}" name="MeasureQty" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{421AF047-51EC-4A36-A9A9-542D272AE863}" name="Unit" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{0D4C0861-5295-4469-9060-36C67ACABC6D}" name="Cost/Unit" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{BBD3AD85-1449-4CE0-A866-53E98118D8FF}" name="MeasureCostOverride" dataDxfId="0"/>
-    <tableColumn id="10" xr3:uid="{8B9D0999-BF75-41B6-BFAF-2393EE709684}" name="Saved kWh" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{87A7CA61-9F27-43F1-83EA-97E23A2B7218}" name="Saved Therms" dataDxfId="15"/>
-    <tableColumn id="12" xr3:uid="{55350E85-083E-4A94-A753-90ADE3A00ADC}" name="Saved MMBTU" dataDxfId="14"/>
-    <tableColumn id="13" xr3:uid="{7D3DBE71-CF6A-427A-8918-CBD299D2FCD2}" name="Deemed kWh" dataDxfId="13"/>
-    <tableColumn id="14" xr3:uid="{C8BFC953-8DC6-420B-A5A3-A9D3DC3F1EFF}" name="Deemed Therms" dataDxfId="12"/>
-    <tableColumn id="15" xr3:uid="{5575EA41-757F-4FF8-8127-80560DDE6A1A}" name="Deemed MMBTU" dataDxfId="11"/>
-    <tableColumn id="16" xr3:uid="{15C99AD5-0ECD-448C-8A28-EED970DC2B47}" name="SavedkWh" dataDxfId="10"/>
-    <tableColumn id="17" xr3:uid="{743920B1-F9D6-49B9-B938-E8706417F532}" name="SavedTherms" dataDxfId="9"/>
-    <tableColumn id="18" xr3:uid="{934FEE5C-80C9-486C-8288-0AE00744E473}" name="SavedMBTUs" dataDxfId="8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DF844518-2BF6-446A-A312-CEB862DCE28B}" name="Table1" displayName="Table1" ref="A1:S11" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23" tableBorderDxfId="22">
+  <autoFilter ref="A1:S11" xr:uid="{DF844518-2BF6-446A-A312-CEB862DCE28B}"/>
+  <tableColumns count="19">
+    <tableColumn id="1" xr3:uid="{1C0006D7-B99F-4704-908A-2CA80F2C4948}" name="AuditId" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{FE306C0E-B210-4780-8F5C-9021F0A2B9A0}" name="ReportingCode" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{8E31AB8D-C308-426E-B4B5-FEDE3ACE3234}" name="Code" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{E78062F7-BD26-4033-A7AE-088E604FD3BA}" name="MeasureQty" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{421AF047-51EC-4A36-A9A9-542D272AE863}" name="Unit" dataDxfId="17"/>
+    <tableColumn id="16" xr3:uid="{15C99AD5-0ECD-448C-8A28-EED970DC2B47}" name="SavedkWh" dataDxfId="16"/>
+    <tableColumn id="19" xr3:uid="{94163277-CD63-4DD0-AE3C-B8EDD0FE1DEE}" name="kW"/>
+    <tableColumn id="17" xr3:uid="{743920B1-F9D6-49B9-B938-E8706417F532}" name="SavedTherms" dataDxfId="15"/>
+    <tableColumn id="18" xr3:uid="{934FEE5C-80C9-486C-8288-0AE00744E473}" name="SavedMBTUs" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{BBD3AD85-1449-4CE0-A866-53E98118D8FF}" name="MeasureCostOverride" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{CC9645AE-FB6D-4AEE-80F7-3A498704D7AE}" name="Measure" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{61A9A28F-0DC7-4361-B3A0-86A213988794}" name="Src" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{0D4C0861-5295-4469-9060-36C67ACABC6D}" name="Cost/Unit" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{8B9D0999-BF75-41B6-BFAF-2393EE709684}" name="Saved kWh" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{87A7CA61-9F27-43F1-83EA-97E23A2B7218}" name="Saved Therms" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{55350E85-083E-4A94-A753-90ADE3A00ADC}" name="Saved MMBTU" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{7D3DBE71-CF6A-427A-8918-CBD299D2FCD2}" name="Deemed kWh" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{C8BFC953-8DC6-420B-A5A3-A9D3DC3F1EFF}" name="Deemed Therms" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{5575EA41-757F-4FF8-8127-80560DDE6A1A}" name="Deemed MMBTU" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -980,8 +1016,8 @@
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{BDEEC43D-CFF6-4115-B5E5-E72781776690}" name="AuditId"/>
     <tableColumn id="2" xr3:uid="{4D6390CE-BE78-4AB7-B4F0-9C26A608BC6F}" name="Fuel"/>
-    <tableColumn id="3" xr3:uid="{5E321DFC-B00C-4D3A-9937-812E28D0C1A4}" name="ElectricBillStartDate" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{4A090723-49F1-49FF-BBAF-9869CC064E4C}" name="ElectricBillEndDate" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{5E321DFC-B00C-4D3A-9937-812E28D0C1A4}" name="ElectricBillStartDate" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{4A090723-49F1-49FF-BBAF-9869CC064E4C}" name="ElectricBillEndDate" dataDxfId="2"/>
     <tableColumn id="5" xr3:uid="{E6903F97-96C0-4DEB-AEA4-0E4CBDCE9A20}" name="Billed Days"/>
     <tableColumn id="6" xr3:uid="{E3938158-341A-4BA4-B0D8-790E5E17FFE3}" name="ElectricMonthkWhUsage"/>
     <tableColumn id="7" xr3:uid="{0D3525C4-6083-4ECF-9898-75775E6C50CE}" name="Units"/>
@@ -997,8 +1033,8 @@
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{FF820CEE-833C-498C-8916-3672D128CC74}" name="AuditId"/>
     <tableColumn id="2" xr3:uid="{81C2C5CE-FB3F-41A7-BE7C-1DA525E3F35D}" name="Fuel"/>
-    <tableColumn id="3" xr3:uid="{3F38A414-1888-4F41-8BB4-20D80742C923}" name="GasBillStartDate" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{E37C4012-C6B6-4607-86E9-C2C8783ADE5B}" name="Gas End" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{3F38A414-1888-4F41-8BB4-20D80742C923}" name="GasBillStartDate" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{E37C4012-C6B6-4607-86E9-C2C8783ADE5B}" name="Gas End" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{E09ED464-9ACE-4853-8CB4-C63C2EA570D4}" name="GasBilledDays"/>
     <tableColumn id="6" xr3:uid="{385B53A2-2457-411F-B4F9-C6C885D3D103}" name="GasMonthThermsUsage"/>
     <tableColumn id="7" xr3:uid="{08EC257A-0641-4CB4-B023-52A5F3A4154A}" name="Units"/>
@@ -1325,20 +1361,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E67B6140-5F6A-4F4C-AA2B-FB00F4AD52CD}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>337908</v>
+      </c>
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2">
+        <v>8.5</v>
       </c>
     </row>
   </sheetData>
@@ -1351,449 +1409,454 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89E4B6A5-B598-4E22-B941-109D7B27EABE}">
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="14.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="16.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="16.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="L1" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H1" s="2" t="s">
+      <c r="M1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="J1" s="2" t="s">
+      <c r="N1" t="s">
         <v>24</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="O1" t="s">
         <v>25</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="P1" t="s">
         <v>26</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="Q1" t="s">
         <v>27</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="R1" t="s">
         <v>28</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="S1" t="s">
         <v>29</v>
       </c>
-      <c r="P1" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
-        <v>337908</v>
-      </c>
-      <c r="B2" s="2" t="s">
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>337908</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="4">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2">
+        <v>183.98963199764</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0.62795096244927995</v>
+      </c>
+      <c r="J2" s="4">
+        <v>1486</v>
+      </c>
+      <c r="K2" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="L2" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F2" s="5">
+      <c r="M2">
+        <v>1486</v>
+      </c>
+      <c r="N2">
+        <v>183.98963199764</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0.62795096244927995</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>337908</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="4">
         <v>1</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="E3" t="s">
         <v>34</v>
       </c>
-      <c r="H2" s="2">
-        <v>1486</v>
-      </c>
-      <c r="I2" s="5">
-        <v>1486</v>
-      </c>
-      <c r="J2" s="2">
-        <v>183.98963199764</v>
-      </c>
-      <c r="K2" s="2">
+      <c r="F3">
         <v>0</v>
       </c>
-      <c r="L2" s="2">
-        <v>0.62795096244927995</v>
-      </c>
-      <c r="P2" s="2">
-        <v>183.98963199764</v>
-      </c>
-      <c r="Q2" s="2">
+      <c r="H3">
         <v>0</v>
       </c>
-      <c r="R2" s="2">
-        <v>0.62795096244927995</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
-        <v>337908</v>
-      </c>
-      <c r="B3" s="2" t="s">
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4">
+        <v>30.5</v>
+      </c>
+      <c r="K3" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="L3" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F3" s="5">
+      <c r="M3">
+        <v>30.5</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>337908</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="4">
         <v>1</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="E4" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="2">
-        <v>30.5</v>
-      </c>
-      <c r="I3" s="5">
-        <v>30.5</v>
-      </c>
-      <c r="J3" s="2">
+      <c r="F4">
         <v>0</v>
       </c>
-      <c r="K3" s="2">
+      <c r="H4">
         <v>0</v>
       </c>
-      <c r="L3" s="2">
+      <c r="I4">
         <v>0</v>
       </c>
-      <c r="P3" s="2">
+      <c r="J4" s="4">
+        <v>1241</v>
+      </c>
+      <c r="K4" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" t="s">
+        <v>31</v>
+      </c>
+      <c r="M4">
+        <v>1241</v>
+      </c>
+      <c r="N4">
         <v>0</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="O4">
         <v>0</v>
       </c>
-      <c r="R3" s="2">
+      <c r="P4">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
-        <v>337908</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="2" t="s">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>337908</v>
+      </c>
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="4">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>40.233279896466897</v>
+      </c>
+      <c r="I5">
+        <v>4.02332798964669</v>
+      </c>
+      <c r="J5" s="4">
+        <v>2854</v>
+      </c>
+      <c r="K5" t="s">
+        <v>40</v>
+      </c>
+      <c r="L5" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="5">
+      <c r="M5">
+        <v>2854</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>40.233279896466897</v>
+      </c>
+      <c r="P5">
+        <v>4.02332798964669</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>337908</v>
+      </c>
+      <c r="B6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="4">
         <v>1</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="E6" t="s">
         <v>34</v>
       </c>
-      <c r="H4" s="2">
-        <v>1241</v>
-      </c>
-      <c r="I4" s="5">
-        <v>1241</v>
-      </c>
-      <c r="J4" s="2">
+      <c r="J6" s="4"/>
+      <c r="K6" t="s">
+        <v>43</v>
+      </c>
+      <c r="L6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>337908</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7" s="4"/>
+      <c r="K7" t="s">
+        <v>43</v>
+      </c>
+      <c r="L7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>337908</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="4">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8">
+        <v>8.4600000000000009</v>
+      </c>
+      <c r="H8">
+        <v>6.81</v>
+      </c>
+      <c r="I8">
+        <v>0.709866</v>
+      </c>
+      <c r="J8" s="4">
+        <v>9.9</v>
+      </c>
+      <c r="K8" t="s">
+        <v>43</v>
+      </c>
+      <c r="L8" t="s">
+        <v>44</v>
+      </c>
+      <c r="M8">
+        <v>9.9</v>
+      </c>
+      <c r="Q8">
+        <v>8.4600000000000009</v>
+      </c>
+      <c r="R8">
+        <v>6.81</v>
+      </c>
+      <c r="S8">
+        <v>0.709866</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>337908</v>
+      </c>
+      <c r="B9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="4">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9">
+        <v>67.2</v>
+      </c>
+      <c r="H9">
         <v>0</v>
       </c>
-      <c r="K4" s="2">
+      <c r="I9">
+        <v>0.22928599999999999</v>
+      </c>
+      <c r="J9" s="4">
+        <v>9.9</v>
+      </c>
+      <c r="K9" t="s">
+        <v>43</v>
+      </c>
+      <c r="L9" t="s">
+        <v>44</v>
+      </c>
+      <c r="M9">
+        <v>9.9</v>
+      </c>
+      <c r="Q9">
+        <v>67.2</v>
+      </c>
+      <c r="R9">
         <v>0</v>
       </c>
-      <c r="L4" s="2">
-        <v>0</v>
-      </c>
-      <c r="P4" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="2">
-        <v>0</v>
-      </c>
-      <c r="R4" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
-        <v>337908</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F5" s="5">
+      <c r="S9">
+        <v>0.22928599999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>337908</v>
+      </c>
+      <c r="B10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="4">
         <v>1</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="E10" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="2">
-        <v>2854</v>
-      </c>
-      <c r="I5" s="5">
-        <v>2854</v>
-      </c>
-      <c r="J5" s="2">
-        <v>0</v>
-      </c>
-      <c r="K5" s="2">
-        <v>40.233279896466897</v>
-      </c>
-      <c r="L5" s="2">
-        <v>4.02332798964669</v>
-      </c>
-      <c r="P5" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="2">
-        <v>40.233279896466897</v>
-      </c>
-      <c r="R5" s="2">
-        <v>4.02332798964669</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
-        <v>337908</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="J10" s="4"/>
+      <c r="K10" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="L10" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F6" s="5">
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>337908</v>
+      </c>
+      <c r="B11" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="4">
         <v>1</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="E11" t="s">
         <v>34</v>
       </c>
-      <c r="I6" s="5"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
-        <v>337908</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="J11" s="4"/>
+      <c r="K11" t="s">
         <v>43</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="L11" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F7" s="5">
-        <v>1</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="I7" s="5"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
-        <v>337908</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" s="5">
-        <v>1</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H8" s="2">
-        <v>9.9</v>
-      </c>
-      <c r="I8" s="5">
-        <v>9.9</v>
-      </c>
-      <c r="M8" s="2">
-        <v>8.4600000000000009</v>
-      </c>
-      <c r="N8" s="2">
-        <v>6.81</v>
-      </c>
-      <c r="O8" s="2">
-        <v>0.709866</v>
-      </c>
-      <c r="P8" s="2">
-        <v>8.4600000000000009</v>
-      </c>
-      <c r="Q8" s="2">
-        <v>6.81</v>
-      </c>
-      <c r="R8" s="2">
-        <v>0.709866</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
-        <v>337908</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F9" s="5">
-        <v>1</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H9" s="2">
-        <v>9.9</v>
-      </c>
-      <c r="I9" s="5">
-        <v>9.9</v>
-      </c>
-      <c r="M9" s="2">
-        <v>67.2</v>
-      </c>
-      <c r="N9" s="2">
-        <v>0</v>
-      </c>
-      <c r="O9" s="2">
-        <v>0.22928599999999999</v>
-      </c>
-      <c r="P9" s="2">
-        <v>67.2</v>
-      </c>
-      <c r="Q9" s="2">
-        <v>0</v>
-      </c>
-      <c r="R9" s="2">
-        <v>0.22928599999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
-        <v>337908</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F10" s="5">
-        <v>1</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="I10" s="5"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
-        <v>337908</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F11" s="5">
-        <v>1</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="I11" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1819,22 +1882,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G1" t="s">
@@ -2180,22 +2243,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D1" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>14</v>
       </c>
       <c r="G1" t="s">

</xml_diff>